<commit_message>
Schedule: Align all course dates, weeks, and Excel spreadsheets with the shifted schedule starting today, Monday 18/05/2026
</commit_message>
<xml_diff>
--- a/Planificacion de la catedra.xlsx
+++ b/Planificacion de la catedra.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="21.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.88671875" customWidth="1" style="6" min="7" max="7"/>
@@ -561,7 +561,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Semana 2: 25/05/2026 (Lunes)</t>
+          <t>Semana 1: 18/05/2026 (Lunes)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Semana 3: 01/06/2026 (Lunes)</t>
+          <t>Semana 2: 25/05/2026 (Lunes)</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Semana 4: 08/06/2026 (Lunes)</t>
+          <t>Semana 3: 01/06/2026 (Lunes)</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Semana 5: 15/06/2026 (Lunes)</t>
+          <t>Semana 4: 08/06/2026 (Lunes)</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Semana 6: 22/06/2026 (Lunes)</t>
+          <t>Semana 5: 15/06/2026 (Lunes)</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Semana 7: 29/06/2026 (Lunes)</t>
+          <t>Semana 6: 22/06/2026 (Lunes)</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Semana 8: 06/07/2026 (Lunes)</t>
+          <t>Semana 7: 29/06/2026 (Lunes)</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Semana 9: 13/07/2026 (Lunes)</t>
+          <t>Semana 8: 06/07/2026 (Lunes)</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Semana 9: 20/07/2026 (Lunes)</t>
+          <t>Semana 9: 13/07/2026 (Lunes)</t>
         </is>
       </c>
       <c r="E11" s="1" t="n"/>
@@ -869,14 +869,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>